<commit_message>
Updates from Claude Code session
</commit_message>
<xml_diff>
--- a/data/raw/COA_Quickbooks_matched.xlsx
+++ b/data/raw/COA_Quickbooks_matched.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Trader\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Trader\accounting_automation\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F06AD386-76B4-4FBA-B287-74A85578BEE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3865FF64-C625-4BAD-AE2F-7ED008BE430E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-195" yWindow="-16320" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30315" yWindow="1515" windowWidth="21600" windowHeight="12735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="emr_payment_types" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1795" uniqueCount="472">
   <si>
     <t>Item</t>
   </si>
@@ -1553,7 +1553,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1860,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1DD643-617D-4F20-AF39-97FC2BE6393F}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -1960,6 +1960,14 @@
         <v>408</v>
       </c>
       <c r="B12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
         <v>409</v>
       </c>
     </row>

</xml_diff>